<commit_message>
New rules about creature types
</commit_message>
<xml_diff>
--- a/cards/CreatureCombatWyl_Creatures.xlsx
+++ b/cards/CreatureCombatWyl_Creatures.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shield\Documents\GitHub\CreatureCombat\cards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39A9B147-63B2-4286-99E3-4933684F22A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D16242C-33C1-4D9A-960D-9387D1F85C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2220" yWindow="3405" windowWidth="23295" windowHeight="13410" activeTab="2" xr2:uid="{A1C39383-539F-404C-8541-3FE92D95158A}"/>
+    <workbookView xWindow="3915" yWindow="0" windowWidth="23295" windowHeight="20985" xr2:uid="{A1C39383-539F-404C-8541-3FE92D95158A}"/>
   </bookViews>
   <sheets>
     <sheet name="Creatures" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="219">
   <si>
     <t>Creature</t>
   </si>
@@ -80,9 +80,6 @@
     <t>Adir Doe</t>
   </si>
   <si>
-    <t>Cervid, Ungulate, Plant</t>
-  </si>
-  <si>
     <t>Forest</t>
   </si>
   <si>
@@ -155,9 +152,6 @@
     <t>Plant</t>
   </si>
   <si>
-    <t>Ungulate</t>
-  </si>
-  <si>
     <t>Birth</t>
   </si>
   <si>
@@ -182,12 +176,6 @@
     <t>Adir Lookout</t>
   </si>
   <si>
-    <t>Arachnid</t>
-  </si>
-  <si>
-    <t>Cervid, Ungulate, Arachnid</t>
-  </si>
-  <si>
     <t>Eyes Peeled</t>
   </si>
   <si>
@@ -221,9 +209,6 @@
     <t>Light</t>
   </si>
   <si>
-    <t>Cervid, Ungulate, Plant, Light</t>
-  </si>
-  <si>
     <t>Light Tail</t>
   </si>
   <si>
@@ -248,9 +233,6 @@
     <t>Poison</t>
   </si>
   <si>
-    <t>Cervid, Ungulate, Plant, Poison</t>
-  </si>
-  <si>
     <t>Poison Moss</t>
   </si>
   <si>
@@ -275,12 +257,6 @@
     <t>Adir Runhart</t>
   </si>
   <si>
-    <t>Avian</t>
-  </si>
-  <si>
-    <t>Cervid, Ungulate, Avian</t>
-  </si>
-  <si>
     <t>Cloud</t>
   </si>
   <si>
@@ -368,9 +344,6 @@
     <t>Undead</t>
   </si>
   <si>
-    <t>Cervid, Ungulate, Poison, Undead</t>
-  </si>
-  <si>
     <t>Wasting</t>
   </si>
   <si>
@@ -395,9 +368,6 @@
     <t>Fire</t>
   </si>
   <si>
-    <t>Avian, Fire</t>
-  </si>
-  <si>
     <t>Volcano</t>
   </si>
   <si>
@@ -446,12 +416,6 @@
     <t>Firefly</t>
   </si>
   <si>
-    <t>Insect</t>
-  </si>
-  <si>
-    <t>Insect, Fire, Light</t>
-  </si>
-  <si>
     <t>Glow</t>
   </si>
   <si>
@@ -467,9 +431,6 @@
     <t>Stone</t>
   </si>
   <si>
-    <t>Avian, Stone</t>
-  </si>
-  <si>
     <t>Lake</t>
   </si>
   <si>
@@ -488,12 +449,6 @@
     <t>Fyrorage</t>
   </si>
   <si>
-    <t>Elemental</t>
-  </si>
-  <si>
-    <t>Fire, Elemental</t>
-  </si>
-  <si>
     <t>Flash Fire</t>
   </si>
   <si>
@@ -509,12 +464,6 @@
     <t>Iguaneous</t>
   </si>
   <si>
-    <t>Reptile</t>
-  </si>
-  <si>
-    <t>Reptile, Stone</t>
-  </si>
-  <si>
     <t>Sunbathe</t>
   </si>
   <si>
@@ -527,9 +476,6 @@
     <t>Lava Grub</t>
   </si>
   <si>
-    <t>Insect, Fire</t>
-  </si>
-  <si>
     <t>Acclimate Volcano</t>
   </si>
   <si>
@@ -539,12 +485,6 @@
     <t>Magma Drake</t>
   </si>
   <si>
-    <t>Dragon</t>
-  </si>
-  <si>
-    <t>Dragon, Fire, Stone</t>
-  </si>
-  <si>
     <t>Fire Breath</t>
   </si>
   <si>
@@ -554,9 +494,6 @@
     <t>Magnimog</t>
   </si>
   <si>
-    <t>Cervid, Ungulate, Fire, Elemental</t>
-  </si>
-  <si>
     <t>Consume Flesh</t>
   </si>
   <si>
@@ -575,9 +512,6 @@
     <t>Armored Shroom</t>
   </si>
   <si>
-    <t>Plant, Stone</t>
-  </si>
-  <si>
     <t>Armor Up</t>
   </si>
   <si>
@@ -587,9 +521,6 @@
     <t>Obsidiax</t>
   </si>
   <si>
-    <t>Insect, Stone, Elemental</t>
-  </si>
-  <si>
     <t>Obsidian Armor</t>
   </si>
   <si>
@@ -605,9 +536,6 @@
     <t>Equine</t>
   </si>
   <si>
-    <t>Equine, Ungulate, Avian, Fire</t>
-  </si>
-  <si>
     <t>Flamebow</t>
   </si>
   <si>
@@ -632,9 +560,6 @@
     <t>Shady Raccoon</t>
   </si>
   <si>
-    <t>Raccoon</t>
-  </si>
-  <si>
     <t>Shady Deal</t>
   </si>
   <si>
@@ -653,18 +578,12 @@
     <t>Moonhowler</t>
   </si>
   <si>
-    <t>Wolf</t>
-  </si>
-  <si>
     <t>Howl Call</t>
   </si>
   <si>
     <t>Vire</t>
   </si>
   <si>
-    <t>Insect, Poison</t>
-  </si>
-  <si>
     <t>Swarm</t>
   </si>
   <si>
@@ -681,6 +600,105 @@
   </si>
   <si>
     <t>We win the game.</t>
+  </si>
+  <si>
+    <t>Cervid, Chiropteran</t>
+  </si>
+  <si>
+    <t>Cervid, Theraphosid</t>
+  </si>
+  <si>
+    <t>Cervid, Plant</t>
+  </si>
+  <si>
+    <t>Cervid, Plant, Light</t>
+  </si>
+  <si>
+    <t>Cervid, Plant, Poison</t>
+  </si>
+  <si>
+    <t>Cervid, Poison, Undead</t>
+  </si>
+  <si>
+    <t>Ramphastid, Fire</t>
+  </si>
+  <si>
+    <t>Phoenicopterid, Stone</t>
+  </si>
+  <si>
+    <t>Canid</t>
+  </si>
+  <si>
+    <t>Theraphosid</t>
+  </si>
+  <si>
+    <t>Chiropteran</t>
+  </si>
+  <si>
+    <t>Phoenicopterid</t>
+  </si>
+  <si>
+    <t>Ramphastid</t>
+  </si>
+  <si>
+    <t>Procyonid</t>
+  </si>
+  <si>
+    <t>Lampyrid</t>
+  </si>
+  <si>
+    <t>Lampyrid, Fire, Light</t>
+  </si>
+  <si>
+    <t>Iguanid</t>
+  </si>
+  <si>
+    <t>Iguanid, Stone</t>
+  </si>
+  <si>
+    <t>Accipitrid</t>
+  </si>
+  <si>
+    <t>Equid, Accipitrid, Fire</t>
+  </si>
+  <si>
+    <t>Lumbricid</t>
+  </si>
+  <si>
+    <t>Lumbricid, Fire</t>
+  </si>
+  <si>
+    <t>Draconid</t>
+  </si>
+  <si>
+    <t>Draconid, Fire, Stone</t>
+  </si>
+  <si>
+    <t>Elementid</t>
+  </si>
+  <si>
+    <t>Cervid, Fire, Elementid</t>
+  </si>
+  <si>
+    <t>Fire, Elementid</t>
+  </si>
+  <si>
+    <t>Polyporiceae</t>
+  </si>
+  <si>
+    <t>Polyporiceae, Stone</t>
+  </si>
+  <si>
+    <t>Scarabaeid</t>
+  </si>
+  <si>
+    <t>Scarabaeid, Stone, Elementid</t>
+  </si>
+  <si>
+    <t>Culicid</t>
+  </si>
+  <si>
+    <t>Culicid, Poison</t>
   </si>
 </sst>
 </file>
@@ -1117,16 +1135,16 @@
         <v>8</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>201</v>
+        <v>176</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="P3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q3" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="R3" s="1" t="s">
         <v>9</v>
@@ -1140,46 +1158,46 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>188</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4">
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G4">
         <v>3</v>
       </c>
       <c r="H4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I4">
         <v>2</v>
       </c>
       <c r="J4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K4">
         <v>-2</v>
       </c>
       <c r="L4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M4">
         <v>-3</v>
       </c>
       <c r="P4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Q4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="R4">
         <v>2</v>
@@ -1190,49 +1208,49 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
         <v>12</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
       </c>
       <c r="E5">
         <v>2</v>
       </c>
       <c r="F5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
         <v>14</v>
       </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
         <v>15</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5" t="s">
-        <v>16</v>
       </c>
       <c r="K5">
         <v>-3</v>
       </c>
       <c r="L5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M5">
         <v>-4</v>
       </c>
       <c r="P5" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q5" t="s">
         <v>38</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>40</v>
       </c>
       <c r="R5">
         <v>1</v>
@@ -1243,49 +1261,49 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>187</v>
       </c>
       <c r="C6">
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6">
         <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G6">
         <v>2</v>
       </c>
       <c r="H6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I6">
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K6">
         <v>-3</v>
       </c>
       <c r="L6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M6">
         <v>-5</v>
       </c>
       <c r="P6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="Q6" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="R6">
         <v>2</v>
@@ -1296,46 +1314,46 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>189</v>
       </c>
       <c r="C7">
         <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E7">
         <v>7</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G7">
         <v>5</v>
       </c>
       <c r="H7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I7">
         <v>4</v>
       </c>
       <c r="J7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K7">
         <v>-1</v>
       </c>
       <c r="L7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M7">
         <v>-2</v>
       </c>
       <c r="P7" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="R7">
         <v>4</v>
@@ -1346,49 +1364,49 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B8" t="s">
-        <v>68</v>
+        <v>190</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8">
         <v>4</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G8">
         <v>3</v>
       </c>
       <c r="H8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I8">
         <v>2</v>
       </c>
       <c r="J8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K8">
         <v>-2</v>
       </c>
       <c r="L8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M8">
         <v>-5</v>
       </c>
       <c r="P8" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="Q8" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="R8">
         <v>3</v>
@@ -1399,49 +1417,49 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>186</v>
       </c>
       <c r="C9">
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E9">
         <v>5</v>
       </c>
       <c r="F9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G9">
         <v>4</v>
       </c>
       <c r="H9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I9">
         <v>3</v>
       </c>
       <c r="J9" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="K9">
         <v>2</v>
       </c>
       <c r="L9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M9">
         <v>-9</v>
       </c>
       <c r="P9" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Q9" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="R9">
         <v>2</v>
@@ -1452,46 +1470,46 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>188</v>
       </c>
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E10">
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G10">
         <v>4</v>
       </c>
       <c r="H10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I10">
         <v>4</v>
       </c>
       <c r="J10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K10">
         <v>-4</v>
       </c>
       <c r="L10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M10">
         <v>-4</v>
       </c>
       <c r="P10" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="R10">
         <v>2</v>
@@ -1502,46 +1520,46 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>188</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E11">
         <v>5</v>
       </c>
       <c r="F11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G11">
         <v>4</v>
       </c>
       <c r="H11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I11">
         <v>4</v>
       </c>
       <c r="J11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K11">
         <v>-5</v>
       </c>
       <c r="L11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M11">
         <v>-7</v>
       </c>
       <c r="P11" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="R11">
         <v>3</v>
@@ -1552,46 +1570,46 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>188</v>
       </c>
       <c r="C12">
         <v>3</v>
       </c>
       <c r="D12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E12">
         <v>4</v>
       </c>
       <c r="F12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G12">
         <v>3</v>
       </c>
       <c r="H12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I12">
         <v>2</v>
       </c>
       <c r="J12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K12">
         <v>-3</v>
       </c>
       <c r="L12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M12">
         <v>-4</v>
       </c>
       <c r="P12" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="R12">
         <v>2</v>
@@ -1602,49 +1620,49 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="B13" t="s">
-        <v>108</v>
+        <v>191</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E13">
         <v>2</v>
       </c>
       <c r="F13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G13">
         <v>-1</v>
       </c>
       <c r="H13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I13">
         <v>-1</v>
       </c>
       <c r="J13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K13">
         <v>-1</v>
       </c>
       <c r="L13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M13">
         <v>-1</v>
       </c>
       <c r="P13" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="Q13" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="R13">
         <v>1</v>
@@ -1655,46 +1673,46 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="B14" t="s">
-        <v>117</v>
+        <v>192</v>
       </c>
       <c r="C14">
         <v>3</v>
       </c>
       <c r="D14" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E14">
         <v>7</v>
       </c>
       <c r="F14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G14">
         <v>5</v>
       </c>
       <c r="H14" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="I14">
         <v>3</v>
       </c>
       <c r="J14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K14">
         <v>-2</v>
       </c>
       <c r="L14" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="M14">
         <v>-7</v>
       </c>
       <c r="P14" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="R14">
         <v>3</v>
@@ -1705,49 +1723,49 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="B15" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E15">
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G15">
         <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="I15">
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="K15">
         <v>-3</v>
       </c>
       <c r="L15" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="M15">
         <v>-7</v>
       </c>
       <c r="P15" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="Q15" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="S15">
         <v>2</v>
@@ -1755,40 +1773,40 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="B16" t="s">
-        <v>135</v>
+        <v>201</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
       <c r="D16" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E16">
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
       <c r="H16" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16" t="s">
         <v>13</v>
       </c>
-      <c r="I16">
-        <v>1</v>
-      </c>
-      <c r="J16" t="s">
-        <v>14</v>
-      </c>
       <c r="K16">
         <v>1</v>
       </c>
       <c r="P16" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="R16">
         <v>2</v>
@@ -1799,46 +1817,46 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="B17" t="s">
-        <v>141</v>
+        <v>193</v>
       </c>
       <c r="C17">
         <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E17">
         <v>5</v>
       </c>
       <c r="F17" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="G17">
         <v>4</v>
       </c>
       <c r="H17" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="I17">
         <v>3</v>
       </c>
       <c r="J17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K17">
         <v>-4</v>
       </c>
       <c r="L17" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="M17">
         <v>-6</v>
       </c>
       <c r="P17" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="R17">
         <v>1</v>
@@ -1849,49 +1867,49 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s">
-        <v>149</v>
+        <v>212</v>
       </c>
       <c r="C18">
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E18">
         <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G18">
         <v>5</v>
       </c>
       <c r="H18" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="I18">
         <v>-5</v>
       </c>
       <c r="J18" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="K18">
         <v>-6</v>
       </c>
       <c r="L18" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="M18">
         <v>-7</v>
       </c>
       <c r="P18" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="Q18" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="R18">
         <v>1</v>
@@ -1902,46 +1920,46 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="B19" t="s">
-        <v>156</v>
+        <v>203</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E19">
         <v>7</v>
       </c>
       <c r="F19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G19">
         <v>4</v>
       </c>
       <c r="H19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I19">
         <v>3</v>
       </c>
       <c r="J19" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="K19">
         <v>-2</v>
       </c>
       <c r="L19" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="M19">
         <v>-3</v>
       </c>
       <c r="P19" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="R19">
         <v>2</v>
@@ -1952,22 +1970,22 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>160</v>
+        <v>143</v>
       </c>
       <c r="B20" t="s">
-        <v>161</v>
+        <v>207</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="P20" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="R20">
         <v>1</v>
@@ -1978,46 +1996,46 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="B21" t="s">
-        <v>166</v>
+        <v>209</v>
       </c>
       <c r="C21">
         <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E21">
         <v>25</v>
       </c>
       <c r="F21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G21">
         <v>15</v>
       </c>
       <c r="H21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I21">
         <v>10</v>
       </c>
       <c r="J21" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="K21">
         <v>7</v>
       </c>
       <c r="L21" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="M21">
         <v>3</v>
       </c>
       <c r="P21" t="s">
-        <v>167</v>
+        <v>147</v>
       </c>
       <c r="R21">
         <v>7</v>
@@ -2028,49 +2046,49 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>169</v>
+        <v>149</v>
       </c>
       <c r="B22" t="s">
-        <v>170</v>
+        <v>211</v>
       </c>
       <c r="C22">
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E22">
         <v>8</v>
       </c>
       <c r="F22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G22">
         <v>5</v>
       </c>
       <c r="H22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I22">
         <v>-1</v>
       </c>
       <c r="J22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K22">
         <v>-1</v>
       </c>
       <c r="L22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M22">
         <v>-1</v>
       </c>
       <c r="P22" t="s">
-        <v>171</v>
+        <v>150</v>
       </c>
       <c r="Q22" t="s">
-        <v>173</v>
+        <v>152</v>
       </c>
       <c r="R22">
         <v>3</v>
@@ -2081,34 +2099,34 @@
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>176</v>
+        <v>155</v>
       </c>
       <c r="B23" t="s">
-        <v>177</v>
+        <v>214</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E23">
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="G23">
         <v>-1</v>
       </c>
       <c r="H23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I23">
         <v>-1</v>
       </c>
       <c r="P23" t="s">
-        <v>178</v>
+        <v>156</v>
       </c>
       <c r="S23">
         <v>2</v>
@@ -2116,49 +2134,49 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
       <c r="B24" t="s">
-        <v>181</v>
+        <v>216</v>
       </c>
       <c r="C24">
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E24">
         <v>5</v>
       </c>
       <c r="F24" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="G24">
         <v>4</v>
       </c>
       <c r="H24" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="I24">
         <v>3</v>
       </c>
       <c r="J24" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="K24">
         <v>-2</v>
       </c>
       <c r="L24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M24">
         <v>-7</v>
       </c>
       <c r="P24" t="s">
-        <v>182</v>
+        <v>159</v>
       </c>
       <c r="Q24" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="R24">
         <v>4</v>
@@ -2169,37 +2187,37 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>185</v>
+        <v>162</v>
       </c>
       <c r="B25" t="s">
-        <v>187</v>
+        <v>205</v>
       </c>
       <c r="C25">
         <v>3</v>
       </c>
       <c r="D25" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E25">
         <v>7</v>
       </c>
       <c r="F25" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="G25">
         <v>4</v>
       </c>
       <c r="H25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I25">
         <v>3</v>
       </c>
       <c r="P25" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="Q25" t="s">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="R25">
         <v>2</v>
@@ -2210,52 +2228,52 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="B26" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C26">
         <v>2</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E26">
         <v>25</v>
       </c>
       <c r="F26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G26">
         <v>15</v>
       </c>
       <c r="H26" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="I26">
         <v>-4</v>
       </c>
       <c r="J26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K26">
         <v>-7</v>
       </c>
       <c r="L26" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M26">
         <v>-15</v>
       </c>
       <c r="N26" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="O26">
         <v>-15</v>
       </c>
       <c r="P26" t="s">
-        <v>197</v>
+        <v>172</v>
       </c>
       <c r="R26">
         <v>1</v>
@@ -2266,46 +2284,46 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>202</v>
+        <v>177</v>
       </c>
       <c r="B27" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="C27">
         <v>5</v>
       </c>
       <c r="D27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E27">
         <v>10</v>
       </c>
       <c r="F27" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="G27">
         <v>9</v>
       </c>
       <c r="H27" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="I27">
         <v>2</v>
       </c>
       <c r="J27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K27">
         <v>-3</v>
       </c>
       <c r="L27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M27">
         <v>-5</v>
       </c>
       <c r="P27" t="s">
-        <v>204</v>
+        <v>178</v>
       </c>
       <c r="R27">
         <v>5</v>
@@ -2316,49 +2334,49 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>205</v>
+        <v>179</v>
       </c>
       <c r="B28" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="E28">
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="G28">
         <v>1</v>
       </c>
       <c r="H28" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="I28">
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="K28">
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M28">
         <v>1</v>
       </c>
       <c r="P28" t="s">
-        <v>207</v>
+        <v>180</v>
       </c>
       <c r="Q28" t="s">
-        <v>208</v>
+        <v>181</v>
       </c>
       <c r="S28">
         <v>1</v>
@@ -2366,49 +2384,49 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>210</v>
+        <v>183</v>
       </c>
       <c r="B29" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E29">
         <v>15</v>
       </c>
       <c r="F29" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="G29">
         <v>-10</v>
       </c>
       <c r="H29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I29">
         <v>-10</v>
       </c>
       <c r="J29" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="K29">
         <v>-10</v>
       </c>
       <c r="L29" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M29">
         <v>-10</v>
       </c>
       <c r="P29" t="s">
-        <v>211</v>
+        <v>184</v>
       </c>
       <c r="Q29" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="R29">
         <v>2</v>
@@ -2461,611 +2479,611 @@
   <sheetData>
     <row r="3" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
         <v>18</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
       <c r="I4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
         <v>31</v>
       </c>
-      <c r="D5" t="s">
+      <c r="I5" t="s">
         <v>32</v>
-      </c>
-      <c r="I5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
         <v>19</v>
       </c>
-      <c r="D6" t="s">
-        <v>20</v>
-      </c>
       <c r="I6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
         <v>40</v>
       </c>
-      <c r="B7" t="s">
+      <c r="G7" t="s">
         <v>41</v>
       </c>
-      <c r="D7" t="s">
+      <c r="I7" t="s">
         <v>42</v>
-      </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I7" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I8" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" t="s">
+        <v>50</v>
+      </c>
+      <c r="I9" t="s">
         <v>52</v>
-      </c>
-      <c r="D9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" t="s">
-        <v>54</v>
-      </c>
-      <c r="I9" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G10" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H10">
         <v>5</v>
       </c>
       <c r="I10" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="I11" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D12" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="I12" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="D13" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="I13" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D14" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="I14" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="D15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I15" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" t="s">
+        <v>89</v>
+      </c>
+      <c r="G16" t="s">
+        <v>56</v>
+      </c>
+      <c r="I16" t="s">
         <v>91</v>
-      </c>
-      <c r="B16" t="s">
-        <v>92</v>
-      </c>
-      <c r="C16" t="s">
-        <v>97</v>
-      </c>
-      <c r="G16" t="s">
-        <v>61</v>
-      </c>
-      <c r="I16" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C17" t="s">
+        <v>89</v>
+      </c>
+      <c r="E17" t="s">
+        <v>96</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="I17" t="s">
         <v>97</v>
-      </c>
-      <c r="E17" t="s">
-        <v>104</v>
-      </c>
-      <c r="F17">
-        <v>1</v>
-      </c>
-      <c r="I17" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="B18" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I18" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="I19" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="B20" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="G20" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="I20" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="I21" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="B22" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C22" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="D22" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="G22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I22" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="B23" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="D23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I23" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="B24" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D24" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="I24" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="B25" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="E25" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
       <c r="G25" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I25" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="B26" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="G26" t="s">
-        <v>189</v>
+        <v>165</v>
       </c>
       <c r="I26" t="s">
-        <v>190</v>
+        <v>166</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="B27" t="s">
-        <v>158</v>
+        <v>141</v>
       </c>
       <c r="D27" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="G27" t="s">
-        <v>159</v>
+        <v>142</v>
       </c>
       <c r="I27" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="D28" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="I28" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>167</v>
+        <v>147</v>
       </c>
       <c r="C29" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="G29" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="I29" t="s">
-        <v>168</v>
+        <v>148</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>171</v>
+        <v>150</v>
       </c>
       <c r="E30" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="F30">
         <v>1</v>
       </c>
       <c r="I30" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>173</v>
+        <v>152</v>
       </c>
       <c r="G31" t="s">
-        <v>174</v>
+        <v>153</v>
       </c>
       <c r="H31">
         <v>10</v>
       </c>
       <c r="I31" t="s">
-        <v>175</v>
+        <v>154</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>178</v>
+        <v>156</v>
       </c>
       <c r="B32" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="D32" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="I32" t="s">
-        <v>179</v>
+        <v>157</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>182</v>
+        <v>159</v>
       </c>
       <c r="B33" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="D33" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="I33" t="s">
-        <v>183</v>
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="B34" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D34" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="I34" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B35" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="E35" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="F35">
         <v>2</v>
       </c>
       <c r="I35" t="s">
-        <v>191</v>
+        <v>167</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="B36" t="s">
-        <v>193</v>
+        <v>169</v>
       </c>
       <c r="D36" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="I36" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>197</v>
+        <v>172</v>
       </c>
       <c r="B37" t="s">
-        <v>198</v>
+        <v>173</v>
       </c>
       <c r="E37" t="s">
-        <v>199</v>
+        <v>174</v>
       </c>
       <c r="F37">
         <v>1</v>
       </c>
       <c r="I37" t="s">
-        <v>200</v>
+        <v>175</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>204</v>
+        <v>178</v>
       </c>
       <c r="B38" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D38" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I38" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>207</v>
+        <v>180</v>
       </c>
       <c r="B39" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G39" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="I39" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>208</v>
+        <v>181</v>
       </c>
       <c r="B40" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D40" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="I40" t="s">
-        <v>209</v>
+        <v>182</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>211</v>
+        <v>184</v>
       </c>
       <c r="B41" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C41" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="D41" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="G41" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="H41">
         <v>20</v>
       </c>
       <c r="I41" t="s">
-        <v>212</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -3111,363 +3129,396 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74E7E971-E9D5-4628-A11F-3D2EB9D9EDB7}">
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>46</v>
+        <v>204</v>
       </c>
       <c r="B1" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="D1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="E1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="F1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G1" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="H1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="J1" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>194</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="E2" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G2" t="s">
-        <v>199</v>
+        <v>174</v>
       </c>
       <c r="H2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
         <v>96</v>
       </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>104</v>
-      </c>
       <c r="H3" t="s">
-        <v>174</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>165</v>
+        <v>196</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="F4" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="H4" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>148</v>
+        <v>217</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="F5" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="H5" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>186</v>
+        <v>208</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="F6" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>116</v>
+        <v>210</v>
       </c>
       <c r="B7" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" t="s">
         <v>31</v>
       </c>
-      <c r="F7" t="s">
-        <v>32</v>
-      </c>
       <c r="H7" t="s">
-        <v>189</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>134</v>
+        <v>163</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F8" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>107</v>
       </c>
       <c r="B9" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="D9" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H9" t="s">
-        <v>159</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F10" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>200</v>
       </c>
       <c r="B11" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="D11" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>196</v>
+        <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F12" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>155</v>
+        <v>206</v>
       </c>
       <c r="D13" t="s">
-        <v>158</v>
+        <v>141</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>126</v>
+        <v>197</v>
       </c>
       <c r="D14" t="s">
-        <v>198</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>140</v>
+        <v>35</v>
       </c>
       <c r="D15" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>107</v>
+        <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>193</v>
+        <v>169</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>213</v>
       </c>
       <c r="D17" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>203</v>
+        <v>199</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>141</v>
+        <v>215</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>195</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>59</v>
+        <v>192</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>68</v>
+        <v>193</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>108</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>187</v>
+        <v>211</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>149</v>
+        <v>188</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>161</v>
+        <v>189</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>135</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>181</v>
+        <v>218</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>127</v>
+        <v>209</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>177</v>
+        <v>205</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>156</v>
+        <v>212</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Creature DNA code stuff
</commit_message>
<xml_diff>
--- a/cards/CreatureCombatWyl_Creatures.xlsx
+++ b/cards/CreatureCombatWyl_Creatures.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shield\Documents\GitHub\CreatureCombat\cards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88736551-53E7-415C-8C45-B84D35152DE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD912D7-B69D-4F24-ADC6-F0DA74A93F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3915" yWindow="5955" windowWidth="23295" windowHeight="13410" activeTab="2" xr2:uid="{A1C39383-539F-404C-8541-3FE92D95158A}"/>
+    <workbookView xWindow="11460" yWindow="1455" windowWidth="17205" windowHeight="13410" activeTab="1" xr2:uid="{A1C39383-539F-404C-8541-3FE92D95158A}"/>
   </bookViews>
   <sheets>
     <sheet name="Creatures" sheetId="1" r:id="rId1"/>
-    <sheet name="Abilities" sheetId="3" r:id="rId2"/>
-    <sheet name="Constants" sheetId="2" r:id="rId3"/>
+    <sheet name="Species" sheetId="4" r:id="rId2"/>
+    <sheet name="Worksheet" sheetId="6" r:id="rId3"/>
+    <sheet name="Abilities" sheetId="3" r:id="rId4"/>
+    <sheet name="Constants" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,14 +36,36 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
+      <xlwcv:version warnBelowVersion="2" setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="292">
   <si>
     <t>Creature</t>
   </si>
@@ -699,6 +722,225 @@
   </si>
   <si>
     <t>Culicid, Poison</t>
+  </si>
+  <si>
+    <t>Creature Code</t>
+  </si>
+  <si>
+    <t>Adir</t>
+  </si>
+  <si>
+    <t>ADIR</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Terrain</t>
+  </si>
+  <si>
+    <t>Terrain Mods</t>
+  </si>
+  <si>
+    <t>Mod</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>Num Bin</t>
+  </si>
+  <si>
+    <t>Mod Bin</t>
+  </si>
+  <si>
+    <t>Combined</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>u</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>j</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>l</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>o</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>q</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>t</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>w</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>z</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>_</t>
+  </si>
+  <si>
+    <t>Character Code</t>
+  </si>
+  <si>
+    <t>DENCJBC9W8</t>
+  </si>
+  <si>
+    <t>Rest</t>
+  </si>
+  <si>
+    <t>Magic Genus</t>
+  </si>
+  <si>
+    <t>Male Code</t>
+  </si>
+  <si>
+    <t>Female Code</t>
+  </si>
+  <si>
+    <t>EMBIRD</t>
+  </si>
+  <si>
+    <t>TGVEFCK4S0</t>
+  </si>
+  <si>
+    <t>fDIR</t>
+  </si>
+  <si>
+    <t>kMBIRD</t>
   </si>
 </sst>
 </file>
@@ -722,12 +964,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -751,7 +999,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -765,6 +1013,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2489,6 +2755,1059 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{846694F0-13EA-45EB-8FCD-012521CFEFC2}">
+  <dimension ref="A3:L5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="3"/>
+    <col min="4" max="4" width="12.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="8"/>
+    <col min="6" max="6" width="9.140625" style="6"/>
+    <col min="9" max="9" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="3" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>220</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="G4" t="s">
+        <v>290</v>
+      </c>
+      <c r="I4" t="str">
+        <f>_xlfn.CONCAT(B4,C4,"U",D4,"U",E4,F4,B4)</f>
+        <v>ADIRBUDENCJBC9W8UASADIR</v>
+      </c>
+      <c r="J4">
+        <f>LEN(I4)</f>
+        <v>23</v>
+      </c>
+      <c r="K4" t="str">
+        <f>_xlfn.CONCAT(B4,C4,"U",D4,"U",E4,F4,G4)</f>
+        <v>ADIRBUDENCJBC9W8UASfDIR</v>
+      </c>
+      <c r="L4">
+        <f>LEN(K4)</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="G5" t="s">
+        <v>291</v>
+      </c>
+      <c r="I5" t="str">
+        <f>_xlfn.CONCAT(B5,C5,"U",D5,"U",E5,F5,B5)</f>
+        <v>EMBIRDCUTGVEFCK4S0UBjEMBIRD</v>
+      </c>
+      <c r="J5">
+        <f>LEN(I5)</f>
+        <v>27</v>
+      </c>
+      <c r="K5" t="str">
+        <f>_xlfn.CONCAT(B5,C5,"U",D5,"U",E5,F5,G5)</f>
+        <v>EMBIRDCUTGVEFCK4S0UBjkMBIRD</v>
+      </c>
+      <c r="L5">
+        <f>LEN(K5)</f>
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B38BA671-2B0B-4B55-9035-C39F4767C75E}">
+  <dimension ref="A3:M24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" customWidth="1"/>
+    <col min="3" max="3" width="7.85546875" style="12" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="7.85546875" style="13" hidden="1" customWidth="1"/>
+    <col min="5" max="12" width="7.85546875" style="12" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4" s="12">
+        <f>IF(ISBLANK(A4),0, _xlfn.XMATCH(A4,Constants!B:B)-1)</f>
+        <v>2</v>
+      </c>
+      <c r="D4" s="13" t="str">
+        <f>DEC2BIN(C4,5)</f>
+        <v>00010</v>
+      </c>
+      <c r="E4" s="12" t="str">
+        <f>_xlfn.CONCAT(IF(B4&gt;=0,"0","1"),DEC2BIN(B4,6))</f>
+        <v>0000101</v>
+      </c>
+      <c r="F4" s="12" t="str">
+        <f>_xlfn.CONCAT(D4,E4)</f>
+        <v>000100000101</v>
+      </c>
+      <c r="G4" s="12" t="str">
+        <f>LEFT(F4,6)</f>
+        <v>000100</v>
+      </c>
+      <c r="H4" s="12" t="str">
+        <f>RIGHT(F4,6)</f>
+        <v>000101</v>
+      </c>
+      <c r="I4" s="12">
+        <f>BIN2DEC(G4)</f>
+        <v>4</v>
+      </c>
+      <c r="J4" s="12">
+        <f>BIN2DEC(H4)</f>
+        <v>5</v>
+      </c>
+      <c r="K4" s="12" t="str" cm="1">
+        <f t="array" ref="K4">IF(I4=0,"",INDEX(Constants!$L:$L,Worksheet!I4))</f>
+        <v>D</v>
+      </c>
+      <c r="L4" s="12" t="str" cm="1">
+        <f t="array" ref="L4">IF(J4=0,"",INDEX(Constants!$L:$L,Worksheet!J4))</f>
+        <v>E</v>
+      </c>
+      <c r="M4" t="str">
+        <f>_xlfn.CONCAT(K4,L4)</f>
+        <v>DE</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="12">
+        <f>IF(ISBLANK(A5),0, _xlfn.XMATCH(A5,Constants!B:B)-1)</f>
+        <v>7</v>
+      </c>
+      <c r="D5" s="13" t="str">
+        <f t="shared" ref="D5:D20" si="0">DEC2BIN(C5,5)</f>
+        <v>00111</v>
+      </c>
+      <c r="E5" s="12" t="str">
+        <f t="shared" ref="E5:E20" si="1">_xlfn.CONCAT(IF(B5&gt;=0,"0","1"),DEC2BIN(B5,6))</f>
+        <v>0000011</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f t="shared" ref="F5:F16" si="2">_xlfn.CONCAT(D5,E5)</f>
+        <v>001110000011</v>
+      </c>
+      <c r="G5" s="12" t="str">
+        <f t="shared" ref="G5:G20" si="3">LEFT(F5,6)</f>
+        <v>001110</v>
+      </c>
+      <c r="H5" s="12" t="str">
+        <f t="shared" ref="H5:H16" si="4">RIGHT(F5,6)</f>
+        <v>000011</v>
+      </c>
+      <c r="I5" s="12">
+        <f t="shared" ref="I5:I16" si="5">BIN2DEC(G5)</f>
+        <v>14</v>
+      </c>
+      <c r="J5" s="12">
+        <f t="shared" ref="J5:J16" si="6">BIN2DEC(H5)</f>
+        <v>3</v>
+      </c>
+      <c r="K5" s="12" t="str" cm="1">
+        <f t="array" ref="K5">IF(I5=0,"",INDEX(Constants!$L:$L,Worksheet!I5))</f>
+        <v>N</v>
+      </c>
+      <c r="L5" s="12" t="str" cm="1">
+        <f t="array" ref="L5">IF(J5=0,"",INDEX(Constants!$L:$L,Worksheet!J5))</f>
+        <v>C</v>
+      </c>
+      <c r="M5" t="str">
+        <f t="shared" ref="M5:M24" si="7">_xlfn.CONCAT(K5,L5)</f>
+        <v>NC</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" s="12">
+        <f>IF(ISBLANK(A6),0, _xlfn.XMATCH(A6,Constants!B:B)-1)</f>
+        <v>5</v>
+      </c>
+      <c r="D6" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00101</v>
+      </c>
+      <c r="E6" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000010</v>
+      </c>
+      <c r="F6" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>001010000010</v>
+      </c>
+      <c r="G6" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>001010</v>
+      </c>
+      <c r="H6" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>000010</v>
+      </c>
+      <c r="I6" s="12">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="J6" s="12">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="K6" s="12" t="str" cm="1">
+        <f t="array" ref="K6">IF(I6=0,"",INDEX(Constants!$L:$L,Worksheet!I6))</f>
+        <v>J</v>
+      </c>
+      <c r="L6" s="12" t="str" cm="1">
+        <f t="array" ref="L6">IF(J6=0,"",INDEX(Constants!$L:$L,Worksheet!J6))</f>
+        <v>B</v>
+      </c>
+      <c r="M6" t="str">
+        <f t="shared" si="7"/>
+        <v>JB</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>-2</v>
+      </c>
+      <c r="C7" s="12">
+        <f>IF(ISBLANK(A7),0, _xlfn.XMATCH(A7,Constants!B:B)-1)</f>
+        <v>1</v>
+      </c>
+      <c r="D7" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00001</v>
+      </c>
+      <c r="E7" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>11111111110</v>
+      </c>
+      <c r="F7" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>0000111111111110</v>
+      </c>
+      <c r="G7" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>000011</v>
+      </c>
+      <c r="H7" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>111110</v>
+      </c>
+      <c r="I7" s="12">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="J7" s="12">
+        <f t="shared" si="6"/>
+        <v>62</v>
+      </c>
+      <c r="K7" s="12" t="str" cm="1">
+        <f t="array" ref="K7">IF(I7=0,"",INDEX(Constants!$L:$L,Worksheet!I7))</f>
+        <v>C</v>
+      </c>
+      <c r="L7" s="12" cm="1">
+        <f t="array" ref="L7">IF(J7=0,"",INDEX(Constants!$L:$L,Worksheet!J7))</f>
+        <v>9</v>
+      </c>
+      <c r="M7" t="str">
+        <f t="shared" si="7"/>
+        <v>C9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>-3</v>
+      </c>
+      <c r="C8" s="12">
+        <f>IF(ISBLANK(A8),0, _xlfn.XMATCH(A8,Constants!B:B)-1)</f>
+        <v>11</v>
+      </c>
+      <c r="D8" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>01011</v>
+      </c>
+      <c r="E8" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>11111111101</v>
+      </c>
+      <c r="F8" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>0101111111111101</v>
+      </c>
+      <c r="G8" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>010111</v>
+      </c>
+      <c r="H8" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>111101</v>
+      </c>
+      <c r="I8" s="12">
+        <f t="shared" si="5"/>
+        <v>23</v>
+      </c>
+      <c r="J8" s="12">
+        <f t="shared" si="6"/>
+        <v>61</v>
+      </c>
+      <c r="K8" s="12" t="str" cm="1">
+        <f t="array" ref="K8">IF(I8=0,"",INDEX(Constants!$L:$L,Worksheet!I8))</f>
+        <v>W</v>
+      </c>
+      <c r="L8" s="12" cm="1">
+        <f t="array" ref="L8">IF(J8=0,"",INDEX(Constants!$L:$L,Worksheet!J8))</f>
+        <v>8</v>
+      </c>
+      <c r="M8" t="str">
+        <f t="shared" si="7"/>
+        <v>W8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9" s="12">
+        <f>IF(ISBLANK(A9),0, _xlfn.XMATCH(A9,Constants!B:B)-1)</f>
+        <v>10</v>
+      </c>
+      <c r="D9" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>01010</v>
+      </c>
+      <c r="E9" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000111</v>
+      </c>
+      <c r="F9" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>010100000111</v>
+      </c>
+      <c r="G9" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>010100</v>
+      </c>
+      <c r="H9" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>000111</v>
+      </c>
+      <c r="I9" s="12">
+        <f t="shared" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="J9" s="12">
+        <f t="shared" si="6"/>
+        <v>7</v>
+      </c>
+      <c r="K9" s="12" t="str" cm="1">
+        <f t="array" ref="K9">IF(I9=0,"",INDEX(Constants!$L:$L,Worksheet!I9))</f>
+        <v>T</v>
+      </c>
+      <c r="L9" s="12" t="str" cm="1">
+        <f t="array" ref="L9">IF(J9=0,"",INDEX(Constants!$L:$L,Worksheet!J9))</f>
+        <v>G</v>
+      </c>
+      <c r="M9" t="str">
+        <f t="shared" si="7"/>
+        <v>TG</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10">
+        <v>5</v>
+      </c>
+      <c r="C10" s="12">
+        <f>IF(ISBLANK(A10),0, _xlfn.XMATCH(A10,Constants!B:B)-1)</f>
+        <v>11</v>
+      </c>
+      <c r="D10" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>01011</v>
+      </c>
+      <c r="E10" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000101</v>
+      </c>
+      <c r="F10" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>010110000101</v>
+      </c>
+      <c r="G10" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>010110</v>
+      </c>
+      <c r="H10" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>000101</v>
+      </c>
+      <c r="I10" s="12">
+        <f t="shared" si="5"/>
+        <v>22</v>
+      </c>
+      <c r="J10" s="12">
+        <f t="shared" si="6"/>
+        <v>5</v>
+      </c>
+      <c r="K10" s="12" t="str" cm="1">
+        <f t="array" ref="K10">IF(I10=0,"",INDEX(Constants!$L:$L,Worksheet!I10))</f>
+        <v>V</v>
+      </c>
+      <c r="L10" s="12" t="str" cm="1">
+        <f t="array" ref="L10">IF(J10=0,"",INDEX(Constants!$L:$L,Worksheet!J10))</f>
+        <v>E</v>
+      </c>
+      <c r="M10" t="str">
+        <f t="shared" si="7"/>
+        <v>VE</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11" s="12">
+        <f>IF(ISBLANK(A11),0, _xlfn.XMATCH(A11,Constants!B:B)-1)</f>
+        <v>3</v>
+      </c>
+      <c r="D11" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00011</v>
+      </c>
+      <c r="E11" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000011</v>
+      </c>
+      <c r="F11" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>000110000011</v>
+      </c>
+      <c r="G11" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>000110</v>
+      </c>
+      <c r="H11" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>000011</v>
+      </c>
+      <c r="I11" s="12">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="J11" s="12">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="K11" s="12" t="str" cm="1">
+        <f t="array" ref="K11">IF(I11=0,"",INDEX(Constants!$L:$L,Worksheet!I11))</f>
+        <v>F</v>
+      </c>
+      <c r="L11" s="12" t="str" cm="1">
+        <f t="array" ref="L11">IF(J11=0,"",INDEX(Constants!$L:$L,Worksheet!J11))</f>
+        <v>C</v>
+      </c>
+      <c r="M11" t="str">
+        <f t="shared" si="7"/>
+        <v>FC</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>-7</v>
+      </c>
+      <c r="C12" s="12">
+        <f>IF(ISBLANK(A12),0, _xlfn.XMATCH(A12,Constants!B:B)-1)</f>
+        <v>5</v>
+      </c>
+      <c r="D12" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00101</v>
+      </c>
+      <c r="E12" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>11111111001</v>
+      </c>
+      <c r="F12" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>0010111111111001</v>
+      </c>
+      <c r="G12" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>001011</v>
+      </c>
+      <c r="H12" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>111001</v>
+      </c>
+      <c r="I12" s="12">
+        <f t="shared" si="5"/>
+        <v>11</v>
+      </c>
+      <c r="J12" s="12">
+        <f t="shared" si="6"/>
+        <v>57</v>
+      </c>
+      <c r="K12" s="12" t="str" cm="1">
+        <f t="array" ref="K12">IF(I12=0,"",INDEX(Constants!$L:$L,Worksheet!I12))</f>
+        <v>K</v>
+      </c>
+      <c r="L12" s="12" cm="1">
+        <f t="array" ref="L12">IF(J12=0,"",INDEX(Constants!$L:$L,Worksheet!J12))</f>
+        <v>4</v>
+      </c>
+      <c r="M12" t="str">
+        <f t="shared" si="7"/>
+        <v>K4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B13">
+        <v>-11</v>
+      </c>
+      <c r="C13" s="12">
+        <f>IF(ISBLANK(A13),0, _xlfn.XMATCH(A13,Constants!B:B)-1)</f>
+        <v>9</v>
+      </c>
+      <c r="D13" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>01001</v>
+      </c>
+      <c r="E13" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>11111110101</v>
+      </c>
+      <c r="F13" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>0100111111110101</v>
+      </c>
+      <c r="G13" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>010011</v>
+      </c>
+      <c r="H13" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>110101</v>
+      </c>
+      <c r="I13" s="12">
+        <f t="shared" si="5"/>
+        <v>19</v>
+      </c>
+      <c r="J13" s="12">
+        <f t="shared" si="6"/>
+        <v>53</v>
+      </c>
+      <c r="K13" s="12" t="str" cm="1">
+        <f t="array" ref="K13">IF(I13=0,"",INDEX(Constants!$L:$L,Worksheet!I13))</f>
+        <v>S</v>
+      </c>
+      <c r="L13" s="12" cm="1">
+        <f t="array" ref="L13">IF(J13=0,"",INDEX(Constants!$L:$L,Worksheet!J13))</f>
+        <v>0</v>
+      </c>
+      <c r="M13" t="str">
+        <f t="shared" si="7"/>
+        <v>S0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C14" s="12">
+        <f>IF(ISBLANK(A14),0, _xlfn.XMATCH(A14,Constants!B:B)-1)</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00000</v>
+      </c>
+      <c r="E14" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000000</v>
+      </c>
+      <c r="F14" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>000000000000</v>
+      </c>
+      <c r="G14" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>000000</v>
+      </c>
+      <c r="H14" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>000000</v>
+      </c>
+      <c r="I14" s="12">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J14" s="12">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="K14" s="12" t="str" cm="1">
+        <f t="array" ref="K14">IF(I14=0,"",INDEX(Constants!$L:$L,Worksheet!I14))</f>
+        <v/>
+      </c>
+      <c r="L14" s="12" t="str" cm="1">
+        <f t="array" ref="L14">IF(J14=0,"",INDEX(Constants!$L:$L,Worksheet!J14))</f>
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C15" s="12">
+        <f>IF(ISBLANK(A15),0, _xlfn.XMATCH(A15,Constants!B:B)-1)</f>
+        <v>0</v>
+      </c>
+      <c r="D15" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00000</v>
+      </c>
+      <c r="E15" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000000</v>
+      </c>
+      <c r="F15" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>000000000000</v>
+      </c>
+      <c r="G15" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>000000</v>
+      </c>
+      <c r="H15" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>000000</v>
+      </c>
+      <c r="I15" s="12">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J15" s="12">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="K15" s="12" t="str" cm="1">
+        <f t="array" ref="K15">IF(I15=0,"",INDEX(Constants!$L:$L,Worksheet!I15))</f>
+        <v/>
+      </c>
+      <c r="L15" s="12" t="str" cm="1">
+        <f t="array" ref="L15">IF(J15=0,"",INDEX(Constants!$L:$L,Worksheet!J15))</f>
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C16" s="12">
+        <f>IF(ISBLANK(A16),0, _xlfn.XMATCH(A16,Constants!B:B)-1)</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00000</v>
+      </c>
+      <c r="E16" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000000</v>
+      </c>
+      <c r="F16" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>000000000000</v>
+      </c>
+      <c r="G16" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>000000</v>
+      </c>
+      <c r="H16" s="12" t="str">
+        <f t="shared" si="4"/>
+        <v>000000</v>
+      </c>
+      <c r="I16" s="12">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J16" s="12">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="K16" s="12" t="str" cm="1">
+        <f t="array" ref="K16">IF(I16=0,"",INDEX(Constants!$L:$L,Worksheet!I16))</f>
+        <v/>
+      </c>
+      <c r="L16" s="12" t="str" cm="1">
+        <f t="array" ref="L16">IF(J16=0,"",INDEX(Constants!$L:$L,Worksheet!J16))</f>
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C17" s="12">
+        <f>IF(ISBLANK(A17),0, _xlfn.XMATCH(A17,Constants!B:B)-1)</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00000</v>
+      </c>
+      <c r="E17" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000000</v>
+      </c>
+      <c r="F17" s="12" t="str">
+        <f t="shared" ref="F17:F20" si="8">_xlfn.CONCAT(D17,E17)</f>
+        <v>000000000000</v>
+      </c>
+      <c r="G17" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>000000</v>
+      </c>
+      <c r="H17" s="12" t="str">
+        <f t="shared" ref="H17:H20" si="9">RIGHT(F17,6)</f>
+        <v>000000</v>
+      </c>
+      <c r="I17" s="12">
+        <f t="shared" ref="I17:I20" si="10">BIN2DEC(G17)</f>
+        <v>0</v>
+      </c>
+      <c r="J17" s="12">
+        <f t="shared" ref="J17:J20" si="11">BIN2DEC(H17)</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="12" t="str" cm="1">
+        <f t="array" ref="K17">IF(I17=0,"",INDEX(Constants!$L:$L,Worksheet!I17))</f>
+        <v/>
+      </c>
+      <c r="L17" s="12" t="str" cm="1">
+        <f t="array" ref="L17">IF(J17=0,"",INDEX(Constants!$L:$L,Worksheet!J17))</f>
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C18" s="12">
+        <f>IF(ISBLANK(A18),0, _xlfn.XMATCH(A18,Constants!B:B)-1)</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00000</v>
+      </c>
+      <c r="E18" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000000</v>
+      </c>
+      <c r="F18" s="12" t="str">
+        <f t="shared" si="8"/>
+        <v>000000000000</v>
+      </c>
+      <c r="G18" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>000000</v>
+      </c>
+      <c r="H18" s="12" t="str">
+        <f t="shared" si="9"/>
+        <v>000000</v>
+      </c>
+      <c r="I18" s="12">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J18" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="K18" s="12" t="str" cm="1">
+        <f t="array" ref="K18">IF(I18=0,"",INDEX(Constants!$L:$L,Worksheet!I18))</f>
+        <v/>
+      </c>
+      <c r="L18" s="12" t="str" cm="1">
+        <f t="array" ref="L18">IF(J18=0,"",INDEX(Constants!$L:$L,Worksheet!J18))</f>
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C19" s="12">
+        <f>IF(ISBLANK(A19),0, _xlfn.XMATCH(A19,Constants!B:B)-1)</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00000</v>
+      </c>
+      <c r="E19" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000000</v>
+      </c>
+      <c r="F19" s="12" t="str">
+        <f t="shared" si="8"/>
+        <v>000000000000</v>
+      </c>
+      <c r="G19" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>000000</v>
+      </c>
+      <c r="H19" s="12" t="str">
+        <f t="shared" si="9"/>
+        <v>000000</v>
+      </c>
+      <c r="I19" s="12">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J19" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="K19" s="12" t="str" cm="1">
+        <f t="array" ref="K19">IF(I19=0,"",INDEX(Constants!$L:$L,Worksheet!I19))</f>
+        <v/>
+      </c>
+      <c r="L19" s="12" t="str" cm="1">
+        <f t="array" ref="L19">IF(J19=0,"",INDEX(Constants!$L:$L,Worksheet!J19))</f>
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C20" s="12">
+        <f>IF(ISBLANK(A20),0, _xlfn.XMATCH(A20,Constants!B:B)-1)</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>00000</v>
+      </c>
+      <c r="E20" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>0000000</v>
+      </c>
+      <c r="F20" s="12" t="str">
+        <f t="shared" si="8"/>
+        <v>000000000000</v>
+      </c>
+      <c r="G20" s="12" t="str">
+        <f t="shared" si="3"/>
+        <v>000000</v>
+      </c>
+      <c r="H20" s="12" t="str">
+        <f t="shared" si="9"/>
+        <v>000000</v>
+      </c>
+      <c r="I20" s="12">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J20" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="K20" s="12" t="str" cm="1">
+        <f t="array" ref="K20">IF(I20=0,"",INDEX(Constants!$L:$L,Worksheet!I20))</f>
+        <v/>
+      </c>
+      <c r="L20" s="12" t="str" cm="1">
+        <f t="array" ref="L20">IF(J20=0,"",INDEX(Constants!$L:$L,Worksheet!J20))</f>
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="M21" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="M22" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="M23" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="M24" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{67097E2E-8D17-4B00-97D5-80E1E6C72F7B}">
+          <x14:formula1>
+            <xm:f>Constants!$B:$B</xm:f>
+          </x14:formula1>
+          <xm:sqref>A1:A1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F31B5ED6-50E6-49F6-AF94-97A4FB211017}">
   <dimension ref="A3:I41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3151,15 +4470,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74E7E971-E9D5-4628-A11F-3D2EB9D9EDB7}">
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>204</v>
       </c>
@@ -3184,8 +4504,11 @@
       <c r="J1" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L1" s="3" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>194</v>
       </c>
@@ -3207,8 +4530,11 @@
       <c r="H2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L2" s="3" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -3230,8 +4556,11 @@
       <c r="H3" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L3" s="3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>196</v>
       </c>
@@ -3250,8 +4579,11 @@
       <c r="H4" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L4" s="3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>217</v>
       </c>
@@ -3270,8 +4602,11 @@
       <c r="H5" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L5" s="3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>208</v>
       </c>
@@ -3284,8 +4619,11 @@
       <c r="F6" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L6" s="3" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>210</v>
       </c>
@@ -3301,8 +4639,11 @@
       <c r="H7" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L7" s="3" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>163</v>
       </c>
@@ -3318,8 +4659,11 @@
       <c r="H8" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L8" s="3" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>107</v>
       </c>
@@ -3335,8 +4679,11 @@
       <c r="H9" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L9" s="3" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>202</v>
       </c>
@@ -3349,8 +4696,11 @@
       <c r="F10" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L10" s="3" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>200</v>
       </c>
@@ -3363,8 +4713,11 @@
       <c r="H11" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L11" s="3" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -3374,175 +4727,376 @@
       <c r="F12" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L12" s="3" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>206</v>
       </c>
       <c r="D13" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L13" s="3" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>197</v>
       </c>
       <c r="D14" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L14" s="3" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>35</v>
       </c>
       <c r="D15" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L15" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>62</v>
       </c>
       <c r="D16" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L16" s="3" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>213</v>
       </c>
       <c r="D17" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L17" s="3" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L18" s="3" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L19" s="3" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L20" s="3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L21" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L22" s="3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L23" s="3" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L24" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L25" s="3" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L26" s="3" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L27" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L28" s="3" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L29" s="3" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L30" s="3" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="L31" s="3" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L32" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L33" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L34" s="3" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L35" s="3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L36" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L37" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L38" s="3" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L39" s="3" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L40" s="3" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L41" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L42" s="3" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="L43" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>216</v>
+      </c>
+      <c r="L44" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L45" s="3" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L46" s="3" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L47" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L48" s="3" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="49" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L49" s="3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="50" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L50" s="3" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="51" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L51" s="3" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="52" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L52" s="3" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="53" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L53" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L54" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L55" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L56" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L57" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L58" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L59" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L60" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L61" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L62" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L63" s="3" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="64" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L64" s="3" t="s">
+        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>